<commit_message>
Modified lead.feature and lead.steps file with additional scenarios along with testdata xlsx file
</commit_message>
<xml_diff>
--- a/src/testdata/data.xlsx
+++ b/src/testdata/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Playwright_Course\PlaywrightCucumberFramework\src\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1F41F8F-B628-4204-BC6B-825BBBD4DBBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D590DD-207E-4599-A2FE-BAFE71F5FA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3DF1D48F-7064-43B5-B4B0-DC020BA99D61}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
   <si>
     <t>TCName</t>
   </si>
@@ -73,13 +73,31 @@
     <t>OpenAI</t>
   </si>
   <si>
-    <t>actualLastname</t>
-  </si>
-  <si>
     <t>Ciara</t>
   </si>
   <si>
     <t>Mary Ciara</t>
+  </si>
+  <si>
+    <t>verify_deletion_of_existing_lead</t>
+  </si>
+  <si>
+    <t>fullname</t>
+  </si>
+  <si>
+    <t>firstname</t>
+  </si>
+  <si>
+    <t>Elizabeth Brown</t>
+  </si>
+  <si>
+    <t>X-ceed inc 99</t>
+  </si>
+  <si>
+    <t>Brown</t>
+  </si>
+  <si>
+    <t>Elizabeth</t>
   </si>
 </sst>
 </file>
@@ -424,7 +442,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -554,6 +572,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -599,10 +628,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -978,18 +1008,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B858FA1-F6C4-4A31-BB4E-D8ACA92F9760}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="48.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44.1796875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.81640625" customWidth="1"/>
+    <col min="6" max="6" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1003,16 +1034,19 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>17</v>
+      <c r="H1" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1024,8 +1058,9 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1039,8 +1074,9 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -1054,8 +1090,9 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -1066,15 +1103,16 @@
       <c r="D5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="2"/>
+      <c r="F5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -1085,14 +1123,39 @@
       <c r="D6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="2"/>
+      <c r="F6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A7" s="2" t="s">
         <v>19</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added API test scenarios
</commit_message>
<xml_diff>
--- a/src/testdata/data.xlsx
+++ b/src/testdata/data.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Playwright_Course\PlaywrightCucumberFramework\src\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D590DD-207E-4599-A2FE-BAFE71F5FA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0156EBD6-65AE-4368-9B85-52BB7AB6181C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3DF1D48F-7064-43B5-B4B0-DC020BA99D61}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="38">
   <si>
     <t>TCName</t>
   </si>
@@ -98,6 +99,42 @@
   </si>
   <si>
     <t>Elizabeth</t>
+  </si>
+  <si>
+    <t>Generate Token and check API Response</t>
+  </si>
+  <si>
+    <t>password123</t>
+  </si>
+  <si>
+    <t>Verify updating booking with token</t>
+  </si>
+  <si>
+    <t>totalprice</t>
+  </si>
+  <si>
+    <t>depositpaid</t>
+  </si>
+  <si>
+    <t>checkin</t>
+  </si>
+  <si>
+    <t>checkout</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>2026-01-01</t>
+  </si>
+  <si>
+    <t>2026-02-01</t>
+  </si>
+  <si>
+    <t>additionalneeds</t>
+  </si>
+  <si>
+    <t>Breakfast</t>
   </si>
 </sst>
 </file>
@@ -442,7 +479,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -572,17 +609,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -628,11 +654,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1008,7 +1036,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B858FA1-F6C4-4A31-BB4E-D8ACA92F9760}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="48.36328125" bestFit="1" customWidth="1"/>
@@ -1018,9 +1046,14 @@
     <col min="6" max="6" width="10.36328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.1796875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1045,8 +1078,23 @@
       <c r="H1" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>36</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1059,8 +1107,13 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1075,8 +1128,13 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
     </row>
-    <row r="4" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -1091,8 +1149,13 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
     </row>
-    <row r="5" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -1111,8 +1174,13 @@
         <v>14</v>
       </c>
       <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
     </row>
-    <row r="6" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -1133,8 +1201,13 @@
       <c r="H6" s="2" t="s">
         <v>18</v>
       </c>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
     </row>
-    <row r="7" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -1156,9 +1229,75 @@
       </c>
       <c r="H7" s="2" t="s">
         <v>22</v>
+      </c>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+    </row>
+    <row r="8" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+    </row>
+    <row r="9" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A9" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3">
+        <v>5400</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6B616B4-21B7-418E-B8FE-FF8950E577B2}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refractored the excel data handling logic in authApi and BookingAPi
</commit_message>
<xml_diff>
--- a/src/testdata/data.xlsx
+++ b/src/testdata/data.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Playwright_Course\PlaywrightCucumberFramework\src\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0156EBD6-65AE-4368-9B85-52BB7AB6181C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95C2DEE3-06EA-4A71-9153-E187AEDCC304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3DF1D48F-7064-43B5-B4B0-DC020BA99D61}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{3DF1D48F-7064-43B5-B4B0-DC020BA99D61}"/>
   </bookViews>
   <sheets>
-    <sheet name="data" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="UI" sheetId="1" r:id="rId1"/>
+    <sheet name="Auth" sheetId="2" r:id="rId2"/>
+    <sheet name="Booking" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="44">
   <si>
     <t>TCName</t>
   </si>
@@ -135,6 +136,24 @@
   </si>
   <si>
     <t>Breakfast</t>
+  </si>
+  <si>
+    <t>Generate Token with invalid user details and check API Response</t>
+  </si>
+  <si>
+    <t>Generate Token with invalid password details and check API Response</t>
+  </si>
+  <si>
+    <t>admin345</t>
+  </si>
+  <si>
+    <t>admin1234</t>
+  </si>
+  <si>
+    <t>Verify updating booking with lastname only</t>
+  </si>
+  <si>
+    <t>Generate Token with blank username and check API Response</t>
   </si>
 </sst>
 </file>
@@ -654,12 +673,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
@@ -1258,7 +1276,7 @@
       <c r="M8" s="3"/>
     </row>
     <row r="9" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B9" s="3"/>
@@ -1275,13 +1293,13 @@
       <c r="I9" s="3">
         <v>5400</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="J9" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="K9" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="5" t="s">
+      <c r="L9" s="4" t="s">
         <v>35</v>
       </c>
       <c r="M9" s="3" t="s">
@@ -1295,9 +1313,168 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6B616B4-21B7-418E-B8FE-FF8950E577B2}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="72.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33115EFF-1E22-4DDA-815C-13D1A147A361}">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="48.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.81640625" customWidth="1"/>
+    <col min="3" max="3" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="3">
+        <v>5400</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="3"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="3"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refractored code to generate report
</commit_message>
<xml_diff>
--- a/src/testdata/data.xlsx
+++ b/src/testdata/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Playwright_Course\PlaywrightCucumberFramework\src\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95C2DEE3-06EA-4A71-9153-E187AEDCC304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A687F74E-69C9-4AEA-AC28-C783FD89C1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{3DF1D48F-7064-43B5-B4B0-DC020BA99D61}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3DF1D48F-7064-43B5-B4B0-DC020BA99D61}"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="1" r:id="rId1"/>

</xml_diff>